<commit_message>
Updated ARE_grids_kan model - 2026-03-03 18:17
</commit_message>
<xml_diff>
--- a/VerveStacks_ARE_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_ARE_grids_kan/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ARE_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE0730CA-E031-4299-AD79-F8391139D2AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{197375F7-1C12-4A45-B434-722F7342BDCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="756" uniqueCount="422">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -349,733 +349,829 @@
     <t>t_pos_andor</t>
   </si>
   <si>
-    <t>p_w24394891_ARE</t>
-  </si>
-  <si>
-    <t>e_w24394891_ARE*</t>
+    <t>p_w24394891-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w24394891-400_ARE*</t>
   </si>
   <si>
     <t>OR</t>
   </si>
   <si>
-    <t>p_w29494113_ARE</t>
-  </si>
-  <si>
-    <t>e_w29494113_ARE*</t>
-  </si>
-  <si>
-    <t>p_w29495157_ARE</t>
-  </si>
-  <si>
-    <t>e_w29495157_ARE*</t>
-  </si>
-  <si>
-    <t>p_w29495366_ARE</t>
-  </si>
-  <si>
-    <t>e_w29495366_ARE*</t>
-  </si>
-  <si>
-    <t>p_w29497443_ARE</t>
-  </si>
-  <si>
-    <t>e_w29497443_ARE*</t>
-  </si>
-  <si>
-    <t>p_w29503687_ARE</t>
-  </si>
-  <si>
-    <t>e_w29503687_ARE*</t>
-  </si>
-  <si>
-    <t>p_w29504119_ARE</t>
-  </si>
-  <si>
-    <t>e_w29504119_ARE*</t>
-  </si>
-  <si>
-    <t>p_w29504133_ARE</t>
-  </si>
-  <si>
-    <t>e_w29504133_ARE*</t>
-  </si>
-  <si>
-    <t>p_w94816851_ARE</t>
-  </si>
-  <si>
-    <t>e_w94816851_ARE*</t>
-  </si>
-  <si>
-    <t>p_w94950807_ARE</t>
-  </si>
-  <si>
-    <t>e_w94950807_ARE*</t>
-  </si>
-  <si>
-    <t>p_w94950821_ARE</t>
-  </si>
-  <si>
-    <t>e_w94950821_ARE*</t>
-  </si>
-  <si>
-    <t>p_w94950847_ARE</t>
-  </si>
-  <si>
-    <t>e_w94950847_ARE*</t>
-  </si>
-  <si>
-    <t>p_w95046328_ARE</t>
-  </si>
-  <si>
-    <t>e_w95046328_ARE*</t>
-  </si>
-  <si>
-    <t>p_w95046332_ARE</t>
-  </si>
-  <si>
-    <t>e_w95046332_ARE*</t>
-  </si>
-  <si>
-    <t>p_w95046953_ARE</t>
-  </si>
-  <si>
-    <t>e_w95046953_ARE*</t>
-  </si>
-  <si>
-    <t>p_w95046964_ARE</t>
-  </si>
-  <si>
-    <t>e_w95046964_ARE*</t>
-  </si>
-  <si>
-    <t>p_w95055625_ARE</t>
-  </si>
-  <si>
-    <t>e_w95055625_ARE*</t>
-  </si>
-  <si>
-    <t>p_w95084771_ARE</t>
-  </si>
-  <si>
-    <t>e_w95084771_ARE*</t>
-  </si>
-  <si>
-    <t>p_w95084776_ARE</t>
-  </si>
-  <si>
-    <t>e_w95084776_ARE*</t>
-  </si>
-  <si>
-    <t>p_w95084793_ARE</t>
-  </si>
-  <si>
-    <t>e_w95084793_ARE*</t>
-  </si>
-  <si>
-    <t>p_w95084794_ARE</t>
-  </si>
-  <si>
-    <t>e_w95084794_ARE*</t>
-  </si>
-  <si>
-    <t>p_w95084799_ARE</t>
-  </si>
-  <si>
-    <t>e_w95084799_ARE*</t>
-  </si>
-  <si>
-    <t>p_w95084816_ARE</t>
-  </si>
-  <si>
-    <t>e_w95084816_ARE*</t>
-  </si>
-  <si>
-    <t>p_w1264942732_ARE</t>
-  </si>
-  <si>
-    <t>e_w1264942732_ARE*</t>
-  </si>
-  <si>
-    <t>p_w95099964_ARE</t>
-  </si>
-  <si>
-    <t>e_w95099964_ARE*</t>
-  </si>
-  <si>
-    <t>p_w95099973_ARE</t>
-  </si>
-  <si>
-    <t>e_w95099973_ARE*</t>
-  </si>
-  <si>
-    <t>p_w301647038_ARE</t>
-  </si>
-  <si>
-    <t>e_w301647038_ARE*</t>
-  </si>
-  <si>
-    <t>p_w132159924_ARE</t>
-  </si>
-  <si>
-    <t>e_w132159924_ARE*</t>
-  </si>
-  <si>
-    <t>p_w132159930_ARE</t>
-  </si>
-  <si>
-    <t>e_w132159930_ARE*</t>
-  </si>
-  <si>
-    <t>p_w132517028_ARE</t>
-  </si>
-  <si>
-    <t>e_w132517028_ARE*</t>
-  </si>
-  <si>
-    <t>p_w149865727_ARE</t>
-  </si>
-  <si>
-    <t>e_w149865727_ARE*</t>
-  </si>
-  <si>
-    <t>p_w173064712_ARE</t>
-  </si>
-  <si>
-    <t>e_w173064712_ARE*</t>
-  </si>
-  <si>
-    <t>p_w174871442_ARE</t>
-  </si>
-  <si>
-    <t>e_w174871442_ARE*</t>
-  </si>
-  <si>
-    <t>p_w181332757_ARE</t>
-  </si>
-  <si>
-    <t>e_w181332757_ARE*</t>
-  </si>
-  <si>
-    <t>p_w181332762_ARE</t>
-  </si>
-  <si>
-    <t>e_w181332762_ARE*</t>
-  </si>
-  <si>
-    <t>p_w181332765_ARE</t>
-  </si>
-  <si>
-    <t>e_w181332765_ARE*</t>
-  </si>
-  <si>
-    <t>p_w181353369_ARE</t>
-  </si>
-  <si>
-    <t>e_w181353369_ARE*</t>
-  </si>
-  <si>
-    <t>p_w181353370_ARE</t>
-  </si>
-  <si>
-    <t>e_w181353370_ARE*</t>
-  </si>
-  <si>
-    <t>p_w181353393_ARE</t>
-  </si>
-  <si>
-    <t>e_w181353393_ARE*</t>
-  </si>
-  <si>
-    <t>p_w181361589_ARE</t>
-  </si>
-  <si>
-    <t>e_w181361589_ARE*</t>
-  </si>
-  <si>
-    <t>p_w181362976_ARE</t>
-  </si>
-  <si>
-    <t>e_w181362976_ARE*</t>
-  </si>
-  <si>
-    <t>p_w200057688_ARE</t>
-  </si>
-  <si>
-    <t>e_w200057688_ARE*</t>
-  </si>
-  <si>
-    <t>p_w1225551111_ARE</t>
-  </si>
-  <si>
-    <t>e_w1225551111_ARE*</t>
-  </si>
-  <si>
-    <t>p_w227922802_ARE</t>
-  </si>
-  <si>
-    <t>e_w227922802_ARE*</t>
-  </si>
-  <si>
-    <t>p_w259874704_ARE</t>
-  </si>
-  <si>
-    <t>e_w259874704_ARE*</t>
-  </si>
-  <si>
-    <t>p_w260963603_ARE</t>
-  </si>
-  <si>
-    <t>e_w260963603_ARE*</t>
-  </si>
-  <si>
-    <t>p_w301651304_ARE</t>
-  </si>
-  <si>
-    <t>e_w301651304_ARE*</t>
-  </si>
-  <si>
-    <t>p_w301663552_ARE</t>
-  </si>
-  <si>
-    <t>e_w301663552_ARE*</t>
-  </si>
-  <si>
-    <t>p_w301663553_ARE</t>
-  </si>
-  <si>
-    <t>e_w301663553_ARE*</t>
-  </si>
-  <si>
-    <t>p_w301690692_ARE</t>
-  </si>
-  <si>
-    <t>e_w301690692_ARE*</t>
-  </si>
-  <si>
-    <t>p_w301715569_ARE</t>
-  </si>
-  <si>
-    <t>e_w301715569_ARE*</t>
-  </si>
-  <si>
-    <t>p_w301911494_ARE</t>
-  </si>
-  <si>
-    <t>e_w301911494_ARE*</t>
-  </si>
-  <si>
-    <t>p_w309146009_ARE</t>
-  </si>
-  <si>
-    <t>e_w309146009_ARE*</t>
-  </si>
-  <si>
-    <t>p_w354337246_ARE</t>
-  </si>
-  <si>
-    <t>e_w354337246_ARE*</t>
-  </si>
-  <si>
-    <t>p_w354337254_ARE</t>
-  </si>
-  <si>
-    <t>e_w354337254_ARE*</t>
-  </si>
-  <si>
-    <t>p_w354339381_ARE</t>
-  </si>
-  <si>
-    <t>e_w354339381_ARE*</t>
-  </si>
-  <si>
-    <t>p_w359425700_ARE</t>
-  </si>
-  <si>
-    <t>e_w359425700_ARE*</t>
-  </si>
-  <si>
-    <t>p_w375827318_ARE</t>
-  </si>
-  <si>
-    <t>e_w375827318_ARE*</t>
-  </si>
-  <si>
-    <t>p_w385901993_ARE</t>
-  </si>
-  <si>
-    <t>e_w385901993_ARE*</t>
-  </si>
-  <si>
-    <t>p_w395805805_ARE</t>
-  </si>
-  <si>
-    <t>e_w395805805_ARE*</t>
-  </si>
-  <si>
-    <t>p_w416954887_ARE</t>
-  </si>
-  <si>
-    <t>e_w416954887_ARE*</t>
-  </si>
-  <si>
-    <t>p_w416954890_ARE</t>
-  </si>
-  <si>
-    <t>e_w416954890_ARE*</t>
-  </si>
-  <si>
-    <t>p_w416981962_ARE</t>
-  </si>
-  <si>
-    <t>e_w416981962_ARE*</t>
-  </si>
-  <si>
-    <t>p_w438419245_ARE</t>
-  </si>
-  <si>
-    <t>e_w438419245_ARE*</t>
-  </si>
-  <si>
-    <t>p_w1264993337_ARE</t>
-  </si>
-  <si>
-    <t>e_w1264993337_ARE*</t>
-  </si>
-  <si>
-    <t>p_w526194855_ARE</t>
-  </si>
-  <si>
-    <t>e_w526194855_ARE*</t>
-  </si>
-  <si>
-    <t>p_w722968894_ARE</t>
-  </si>
-  <si>
-    <t>e_w722968894_ARE*</t>
-  </si>
-  <si>
-    <t>p_w801739686_ARE</t>
-  </si>
-  <si>
-    <t>e_w801739686_ARE*</t>
-  </si>
-  <si>
-    <t>p_w900165939_ARE</t>
-  </si>
-  <si>
-    <t>e_w900165939_ARE*</t>
-  </si>
-  <si>
-    <t>p_w939814405_ARE</t>
-  </si>
-  <si>
-    <t>e_w939814405_ARE*</t>
-  </si>
-  <si>
-    <t>p_w1078341293_ARE</t>
-  </si>
-  <si>
-    <t>e_w1078341293_ARE*</t>
-  </si>
-  <si>
-    <t>p_w1168317384_ARE</t>
-  </si>
-  <si>
-    <t>e_w1168317384_ARE*</t>
-  </si>
-  <si>
-    <t>p_w1168317387_ARE</t>
-  </si>
-  <si>
-    <t>e_w1168317387_ARE*</t>
-  </si>
-  <si>
-    <t>p_w1225109215_ARE</t>
-  </si>
-  <si>
-    <t>e_w1225109215_ARE*</t>
-  </si>
-  <si>
-    <t>p_w1242347420_ARE</t>
-  </si>
-  <si>
-    <t>e_w1242347420_ARE*</t>
-  </si>
-  <si>
-    <t>p_w1255406048_ARE</t>
-  </si>
-  <si>
-    <t>e_w1255406048_ARE*</t>
-  </si>
-  <si>
-    <t>p_w1264973879_ARE</t>
-  </si>
-  <si>
-    <t>e_w1264973879_ARE*</t>
-  </si>
-  <si>
-    <t>p_w1348312852_ARE</t>
-  </si>
-  <si>
-    <t>e_w1348312852_ARE*</t>
-  </si>
-  <si>
-    <t>p_w1366982708_ARE</t>
-  </si>
-  <si>
-    <t>e_w1366982708_ARE*</t>
-  </si>
-  <si>
-    <t>p_w1366988951_ARE</t>
-  </si>
-  <si>
-    <t>e_w1366988951_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE5_ARE</t>
-  </si>
-  <si>
-    <t>e_AE5_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE6_ARE</t>
-  </si>
-  <si>
-    <t>e_AE6_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE4_ARE</t>
-  </si>
-  <si>
-    <t>e_AE4_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE3_ARE</t>
-  </si>
-  <si>
-    <t>e_AE3_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE23_ARE</t>
-  </si>
-  <si>
-    <t>e_AE23_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE39_ARE</t>
-  </si>
-  <si>
-    <t>e_AE39_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE33_ARE</t>
-  </si>
-  <si>
-    <t>e_AE33_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE8_ARE</t>
-  </si>
-  <si>
-    <t>e_AE8_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE29_ARE</t>
-  </si>
-  <si>
-    <t>e_AE29_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE37_ARE</t>
-  </si>
-  <si>
-    <t>e_AE37_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE31_ARE</t>
-  </si>
-  <si>
-    <t>e_AE31_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE41_ARE</t>
-  </si>
-  <si>
-    <t>e_AE41_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE36_ARE</t>
-  </si>
-  <si>
-    <t>e_AE36_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE35_ARE</t>
-  </si>
-  <si>
-    <t>e_AE35_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE10_ARE</t>
-  </si>
-  <si>
-    <t>e_AE10_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE22_ARE</t>
-  </si>
-  <si>
-    <t>e_AE22_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE42_ARE</t>
-  </si>
-  <si>
-    <t>e_AE42_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE30_ARE</t>
-  </si>
-  <si>
-    <t>e_AE30_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE19_ARE</t>
-  </si>
-  <si>
-    <t>e_AE19_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE40_ARE</t>
-  </si>
-  <si>
-    <t>e_AE40_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE13_ARE</t>
-  </si>
-  <si>
-    <t>e_AE13_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE2_ARE</t>
-  </si>
-  <si>
-    <t>e_AE2_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE12_ARE</t>
-  </si>
-  <si>
-    <t>e_AE12_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE38_ARE</t>
-  </si>
-  <si>
-    <t>e_AE38_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE11_ARE</t>
-  </si>
-  <si>
-    <t>e_AE11_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE7_ARE</t>
-  </si>
-  <si>
-    <t>e_AE7_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE21_ARE</t>
-  </si>
-  <si>
-    <t>e_AE21_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE24_ARE</t>
-  </si>
-  <si>
-    <t>e_AE24_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE25_ARE</t>
-  </si>
-  <si>
-    <t>e_AE25_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE28_ARE</t>
-  </si>
-  <si>
-    <t>e_AE28_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE26_ARE</t>
-  </si>
-  <si>
-    <t>e_AE26_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE18_ARE</t>
-  </si>
-  <si>
-    <t>e_AE18_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE27_ARE</t>
-  </si>
-  <si>
-    <t>e_AE27_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE1_ARE</t>
-  </si>
-  <si>
-    <t>e_AE1_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE14_ARE</t>
-  </si>
-  <si>
-    <t>e_AE14_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE17_ARE</t>
-  </si>
-  <si>
-    <t>e_AE17_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE34_ARE</t>
-  </si>
-  <si>
-    <t>e_AE34_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE32_ARE</t>
-  </si>
-  <si>
-    <t>e_AE32_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE20_ARE</t>
-  </si>
-  <si>
-    <t>e_AE20_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE15_ARE</t>
-  </si>
-  <si>
-    <t>e_AE15_ARE*</t>
-  </si>
-  <si>
-    <t>p_AE9_ARE</t>
-  </si>
-  <si>
-    <t>e_AE9_ARE*</t>
+    <t>p_w24394891-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w24394891-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w29494113-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w29494113-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w29495157-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w29495157-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w29495366-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w29495366-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w29497443-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w29497443-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w29503687-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w29503687-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w29504119-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w29504119-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w29504119-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w29504119-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w29504133-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w29504133-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w94816851-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w94816851-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w94950807-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w94950807-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w94950821-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w94950821-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w94950847-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w94950847-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w95046328-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w95046328-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w95046332-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w95046332-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w95046953-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w95046953-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w95046953-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w95046953-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w95046964-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w95046964-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w95055625-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w95055625-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w95084771-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w95084771-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w95084776-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w95084776-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w95084793-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w95084793-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w95084794-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w95084794-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w95084799-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w95084799-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w95084799-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w95084799-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w95084816-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w95084816-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w1264942732-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w1264942732-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w95099964-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w95099964-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w95099964-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w95099964-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w95099973-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w95099973-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w301647038-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w301647038-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w301647038-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w301647038-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w132159924-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w132159924-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w132159930-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w132159930-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w132517028-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w132517028-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w149865727-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w149865727-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w173064712-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w173064712-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w174871442-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w174871442-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w181332757-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w181332757-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w181332762-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w181332762-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w181332765-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w181332765-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w181353369-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w181353369-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w181353370-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w181353370-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w181353393-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w181353393-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w181361589-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w181361589-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w181362976-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w181362976-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w200057688-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w200057688-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w200057688-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w200057688-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w1225551111-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w1225551111-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w227922802-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w227922802-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w259874704-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w259874704-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w259874704-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w259874704-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w260963603-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w260963603-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w301651304-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w301651304-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w301663552-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w301663552-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w301663553-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w301663553-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w301690692-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w301690692-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w301715569-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w301715569-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w301911494-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w301911494-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w309146009-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w309146009-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w354337246-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w354337246-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w354337254-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w354337254-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w354337254-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w354337254-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w354339381-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w354339381-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w359425700-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w359425700-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w375827318-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w375827318-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w385901993-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w385901993-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w395805805-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w395805805-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w416954887-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w416954887-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w416954890-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w416954890-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w416981962-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w416981962-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w438419245-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w438419245-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w1264993337-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w1264993337-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w526194855-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w526194855-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w722968894-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w722968894-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w801739686-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w801739686-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w900165939-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w900165939-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w939814405-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w939814405-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w1078341293-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w1078341293-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w1168317384-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w1168317384-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w1168317387-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w1168317387-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w1225109215-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w1225109215-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w1242347420-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w1242347420-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w1255406048-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w1255406048-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w1264973879-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w1264973879-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w526194855-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w526194855-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w1348312852-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w1348312852-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w1366982708-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w1366982708-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w1366988951-400_ARE</t>
+  </si>
+  <si>
+    <t>e_w1366988951-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_w1366988951-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w1366988951-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE5-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE5-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE6-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE6-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE4-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE4-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE3-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE3-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE23-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE23-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE39-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE39-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE33-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE33-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE8-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE8-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE29-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE29-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE37-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE37-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE33-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE33-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE31-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE31-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE41-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE41-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE36-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE36-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE35-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE35-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE10-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE10-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE22-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE22-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE42-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE42-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE30-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE30-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE19-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE19-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE40-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE40-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE13-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE13-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE2-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE2-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE12-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE12-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE38-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE38-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE11-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE11-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE7-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE7-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE21-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE21-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE24-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE24-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE25-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE25-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE28-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE28-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE26-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE26-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE29-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE29-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE19-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE19-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE18-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE18-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE27-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE27-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE1-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE1-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_w354339381-220_ARE</t>
+  </si>
+  <si>
+    <t>e_w354339381-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE14-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE14-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE17-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE17-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE18-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE18-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE34-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE34-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE32-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE32-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE20-220_ARE</t>
+  </si>
+  <si>
+    <t>e_AE20-220_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE15-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE15-400_ARE*</t>
+  </si>
+  <si>
+    <t>p_AE9-400_ARE</t>
+  </si>
+  <si>
+    <t>e_AE9-400_ARE*</t>
   </si>
   <si>
     <t>rez_spv_ARE_001</t>
@@ -2045,8 +2141,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19D09CFA-EE7E-4439-8EF8-A44516A3A252}">
-  <dimension ref="B9:E153"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D65D11E8-2B0C-4700-9A7A-4D9FB5BC6181}">
+  <dimension ref="B9:E169"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
@@ -4067,6 +4163,230 @@
         <v>389</v>
       </c>
       <c r="E153" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="154" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B154" t="s">
+        <v>390</v>
+      </c>
+      <c r="C154" t="s">
+        <v>391</v>
+      </c>
+      <c r="D154" t="s">
+        <v>391</v>
+      </c>
+      <c r="E154" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="155" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B155" t="s">
+        <v>392</v>
+      </c>
+      <c r="C155" t="s">
+        <v>393</v>
+      </c>
+      <c r="D155" t="s">
+        <v>393</v>
+      </c>
+      <c r="E155" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="156" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B156" t="s">
+        <v>394</v>
+      </c>
+      <c r="C156" t="s">
+        <v>395</v>
+      </c>
+      <c r="D156" t="s">
+        <v>395</v>
+      </c>
+      <c r="E156" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="157" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B157" t="s">
+        <v>396</v>
+      </c>
+      <c r="C157" t="s">
+        <v>397</v>
+      </c>
+      <c r="D157" t="s">
+        <v>397</v>
+      </c>
+      <c r="E157" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="158" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B158" t="s">
+        <v>398</v>
+      </c>
+      <c r="C158" t="s">
+        <v>399</v>
+      </c>
+      <c r="D158" t="s">
+        <v>399</v>
+      </c>
+      <c r="E158" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="159" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B159" t="s">
+        <v>400</v>
+      </c>
+      <c r="C159" t="s">
+        <v>401</v>
+      </c>
+      <c r="D159" t="s">
+        <v>401</v>
+      </c>
+      <c r="E159" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="160" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B160" t="s">
+        <v>402</v>
+      </c>
+      <c r="C160" t="s">
+        <v>403</v>
+      </c>
+      <c r="D160" t="s">
+        <v>403</v>
+      </c>
+      <c r="E160" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="161" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B161" t="s">
+        <v>404</v>
+      </c>
+      <c r="C161" t="s">
+        <v>405</v>
+      </c>
+      <c r="D161" t="s">
+        <v>405</v>
+      </c>
+      <c r="E161" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="162" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B162" t="s">
+        <v>406</v>
+      </c>
+      <c r="C162" t="s">
+        <v>407</v>
+      </c>
+      <c r="D162" t="s">
+        <v>407</v>
+      </c>
+      <c r="E162" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="163" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B163" t="s">
+        <v>408</v>
+      </c>
+      <c r="C163" t="s">
+        <v>409</v>
+      </c>
+      <c r="D163" t="s">
+        <v>409</v>
+      </c>
+      <c r="E163" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="164" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B164" t="s">
+        <v>410</v>
+      </c>
+      <c r="C164" t="s">
+        <v>411</v>
+      </c>
+      <c r="D164" t="s">
+        <v>411</v>
+      </c>
+      <c r="E164" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="165" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B165" t="s">
+        <v>412</v>
+      </c>
+      <c r="C165" t="s">
+        <v>413</v>
+      </c>
+      <c r="D165" t="s">
+        <v>413</v>
+      </c>
+      <c r="E165" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="166" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B166" t="s">
+        <v>414</v>
+      </c>
+      <c r="C166" t="s">
+        <v>415</v>
+      </c>
+      <c r="D166" t="s">
+        <v>415</v>
+      </c>
+      <c r="E166" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="167" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B167" t="s">
+        <v>416</v>
+      </c>
+      <c r="C167" t="s">
+        <v>417</v>
+      </c>
+      <c r="D167" t="s">
+        <v>417</v>
+      </c>
+      <c r="E167" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="168" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B168" t="s">
+        <v>418</v>
+      </c>
+      <c r="C168" t="s">
+        <v>419</v>
+      </c>
+      <c r="D168" t="s">
+        <v>419</v>
+      </c>
+      <c r="E168" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="169" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B169" t="s">
+        <v>420</v>
+      </c>
+      <c r="C169" t="s">
+        <v>421</v>
+      </c>
+      <c r="D169" t="s">
+        <v>421</v>
+      </c>
+      <c r="E169" t="s">
         <v>105</v>
       </c>
     </row>

</xml_diff>